<commit_message>
Added NEXUS Board Strategy Comm tracker sheet
</commit_message>
<xml_diff>
--- a/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
+++ b/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
@@ -9,14 +9,15 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Rollout" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feishu Files" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Webinar #1 Tracker" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEXUS Board Strategy Comm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Webinar #1 Tracker" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +74,37 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Crimson Pro"/>
+      <b val="1"/>
+      <color rgb="000F1115"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="DM Sans"/>
+      <color rgb="008A8F9A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="DM Sans"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="IBM Plex Mono"/>
+      <b val="1"/>
+      <color rgb="008A8F9A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="DM Sans"/>
+      <b val="1"/>
+      <color rgb="00D4AC0D"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -153,8 +183,20 @@
         <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F3"/>
+        <bgColor rgb="00F5F5F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBEB"/>
+        <bgColor rgb="00FFFBEB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -196,11 +238,25 @@
         <color rgb="00D0D3D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E0E2E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E0E2E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E2E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E2E6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -259,6 +315,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2010,6 +2075,356 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue Stream</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Pax/Session</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Revenue</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Webinar (free funnel)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>3/month total</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>$0 (lead gen)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Immediate</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Feeds into workshops</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>China &amp; Leadership Workshop</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>$150 / 1000RMB pax</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>3/month</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>5-15 pax</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>$450-$1,350</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Immediate</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Paid, highest volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Career Workshop</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>$150 / 1000RMB pax</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2/month</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>5-15 pax</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>$300-$900</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Immediate</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Leadership Workshop</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>$150 / 1000RMB pax</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1/month</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>5-15 pax</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>$150-$450</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Paid, starts later</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Diagnostic Session</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>$1,000/session</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Post-workshop upsell</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Executive Search</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Project fee</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Signal-triggered</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Highest value per deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL (workshops)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>$900-$2,700 (Oct+)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>$750-$2,250 (Aug-Sep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>6-MO TOTAL</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>$8,100-$24,300</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Plus diagnostics + exec search</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3899,6 +4314,402 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>NEXUS Board — Strategy Communication Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Tracks board-level decisions and communication for NEXUS strategy rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Board strategy review meeting</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Board + Kevin</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Board review of NEXUS strategy direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Board approval of strategy pivot</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Formal board approval for strategy changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Board communication to NEXUS team</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Board + Kevin</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>How strategy is communicated to the NEXUS team</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Board communication to investors</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Board + Kevin</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>Investor-facing strategy update</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>Board communication to market</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Board + Maria/ECHO</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>External market-facing strategy announcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>EXEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Brand rollout alignment with board strategy</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Emily + Kevin</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Aug 12</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Ensure brand rollout is consistent with board-approved strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>NEXUS product roadmap alignment</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>James + Board</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>Product roadmap reflects strategy direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>KPIs / success metrics alignment</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>LENS + Board</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>Define what success looks like post-strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>Risk assessment of strategy shift</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>Hans + Board</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>Identify risks in strategy communication and execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>Client communication plan</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>Maria + Board</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>How to communicate strategy changes to clients</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5003,7 +5814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5483,7 +6294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5832,7 +6643,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6837,7 +7648,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7333,7 +8144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8024,354 +8835,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue Stream</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Frequency</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Pax/Session</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Monthly Revenue</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Webinar (free funnel)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>3/month total</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>$0 (lead gen)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Immediate</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Feeds into workshops</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>China &amp; Leadership Workshop</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>$150 / 1000RMB pax</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>3/month</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>5-15 pax</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>$450-$1,350</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Immediate</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Paid, highest volume</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Career Workshop</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>$150 / 1000RMB pax</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2/month</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>5-15 pax</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>$300-$900</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Immediate</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>AI &amp; Leadership Workshop</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>$150 / 1000RMB pax</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>1/month</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>5-15 pax</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>$150-$450</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Oct 2026</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Paid, starts later</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Diagnostic Session</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>$1,000/session</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>As needed</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Post-workshop upsell</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Executive Search</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Project fee</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Signal-triggered</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Highest value per deal</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL (workshops)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>$900-$2,700 (Oct+)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>$750-$2,250 (Aug-Sep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>6-MO TOTAL</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>$8,100-$24,300</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Plus diagnostics + exec search</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Reorder sheets: Brand Rollout, Webinar #1, NEXUS Board Strategy Comm
</commit_message>
<xml_diff>
--- a/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
+++ b/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
@@ -8,16 +8,16 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Rollout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feishu Files" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Webinar #1 Tracker" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEXUS Board Strategy Comm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Webinar #1 Tracker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feishu Files" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2075,6 +2075,699 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>File Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>webinar_definitions.json</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Event Data</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>29 industry x geo webinar cluster definitions</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>webinar_programs.json</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Event Data</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Program definitions with matching rules, tier assignments</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Automation_Spec_v1.md</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Spec</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Automation specification for Carl workflows</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Density_Clustering_Report_v1.md</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Contact density clustering analysis</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Density_Clustering_Report_v2.md</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Updated density clustering</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Cross_Cluster_Mapping_Report_v1.md</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Cross-cluster contact mapping</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Strategic_Priority_DeepDive_v1.md</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Strategic priority deep-dive</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Subsegmentation_Report_v1.md</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Contact subsegmentation analysis</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>LYC_Content_Pillars_Aligned_v2.xlsx</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Source Excel for Feishu Content Pillars v3</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>LYC_WEEK1_SCRIPTS_V2_FULL.md</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Week 1 v2 complete scripts (~22,403 words)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>headline_scripts_v2_final.json</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Week 1 v2 scripts JSON</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>LYC_YOUTUBE_SCRIPTS_V7_ALL_18_HOOKS_COMPLETE.md</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Series A complete scripts</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>LYC_YOUTUBE_V8_TONE_REVISED.md</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Series B complete scripts</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>LYC_YOUTUBE_HOOK_MAP_V7_BEYOND_HEADLINES.md</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Hook Map</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Series C hook map</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>LYC_YOUTUBE_HOOK_MAP_V10_AI_CAREER.md</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hook Map</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Series D hook map</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Full_Inventory.md</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Complete Carl asset inventory (Markdown)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CARL_Supabase_Tables_Spec.md</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Supabase table specs + workflows</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>WAVE_Project_PM_Tracker.xlsx</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>PM Tracker</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>WAVE project management - 87 tickets with status</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>WAVE_Project/Business_Specs/</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>WAVE business specs (BRD, tickets, intelligence, funnel)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>WAVE_Project/Database_Schema/</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>DB Schema</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Outreach funnel SQL schema</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>WAVE_Project/wave-app/</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Source Code</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Next.js source code for WAVE app (Phase 0)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LYC_Social_Content_Tracker_v1.xlsx</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Social Media Tracker</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>./</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LYC_Social_Content_Tracker_v1.1.xlsx</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Social content tracker — 5 sheets, 26 tasks, 17 formats</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>social_content_playbook_v1.1.docx</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Full social playbook v1.1 with B2B differentiation research</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>emily_social_content_onboarding.docx</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Emily onboarding guide</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>carl_agent_spec_v2.docx</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Agent Identity</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Carl agent spec v2 — dual role (WAVE + content ops)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>/app/data/sessions/session/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2419,7 +3112,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3186,1124 +3879,6 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A33:G33"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="53" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="53" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Document Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Feishu Link</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Content Pillar</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Content Pillars Aligned v3</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/sheets/VDkPsNGEwhmLa4tqA9pcatHNnEh</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Content Calendar</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Master calendar - 3 webinars/mo + workshops by pillar</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Headline-First System v2</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/sheets/OBsMsiX4ThazS1t3ZveczT9inrh</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Content System</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>15 hooks x 3 formats (long/short/reel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Week 1 Scripts v2</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/D2dBdUYMyoIaJSxwULvcR4cFnkd</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>ECHO v4.0 compliant</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>45 scripts (15 hooks x 3), ~22,403 words</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Series A v7</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/Jq8wdU4xloiJAmxHy1wcIDp4n7d</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Career</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>18 hooks, 54 scripts</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Series B v8</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/VYcZdgCOCoh6hgxQjRFc8lvKnjd</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Career</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Tone revised</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>24 hooks, 72 scripts</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Series C Hook Map v7</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/LvWqd4514oBRK7xKmx4c3dX9nZe</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Hook Map</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>China &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>25 hooks, 5 clusters</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Series C Sample Scripts v9</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/ZuCIdAQEDoyeiQxmwoGcdXtanJV</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>China &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>4 samples done</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>4 sample scripts; full 75 pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Series D Hook Map v10</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/VpFJdD1iQoPO9Lxt86Ic8QKpn4e</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Hook Map</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>AI &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>25 hooks, 5 clusters</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Series D Sample Scripts v10</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/VabodDdjJo9eO8xRGFEcrFe6nbc</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>AI &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>4 samples done</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>4 sample scripts; full 75 pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Content Calendar v1 (legacy)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/sheets/XgKrsJNJyhiq6At2ebxc62IAnFR</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Content Calendar</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Superseded by v3</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Original calendar before pillar alignment</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>WAVE BRD v1.0</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/NsrodeH2doEWwMx67fCcT8Xtncc</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Business Requirements Document - 8 modules, 87 tickets</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>WAVE Development Tickets v1.0</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/OLuLdFDWdofvXzxRYCWce2gXnGd</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>87 dev tickets with priority/effort/deps</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>WAVE Intelligence Layer Spec v1.0</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/AqQSdPFxMoXmsyx1LRbcVqAgnqb</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Intelligence module specification</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>LYC Intelligence Design Spec</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/JaczdojEQo7NCBxeoqJco2Ylnod</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Intelligence design specification</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Outreach Funnel Refined v2</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/KNjedt5jsoUWkfxF7Q1cJL8jnuf</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Outreach funnel v2 refined spec</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Outreach Funnel Mapping Spec</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/PyYPdvoj5oy80FxZgPOcpUhNn5d</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>Outreach funnel mapping specification</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>WAVE DB Schema - Outreach Funnel</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Doc</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/CcQTdIh8FoO5YqxKpUXcvSS4n5b</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Database schema SQL for outreach funnel</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>WAVE Project PM Tracker</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>(uploaded file - GaHfbAhjPoF0Z5xUX49ca0mLnnM)</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>87 tickets with status/priority/module tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>WAVE Business Spec Pitch ICP</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Slides</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>(uploaded file - Qye0bsFr5oNzEDx6Oq4c8gnunHg)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>WAVE</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Business pitch deck for ICP</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>ECHO Asset Master v6.0</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Doc (Notion)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>https://lyc-partners.notion.site/ECHO-Asset-Master-v6-0-Source-of-Truth-2026-08-04-3b2fafae51be81aeb291ec9c33e67faa</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Brand Compliance</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Echo</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Source of Truth</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Brand compliance source of truth - designated by Kevin 2026-08-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Social Content Tracker v1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>File (xlsx)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/Nmu4bW4SCoxjjcxMo5pca1N3nPg</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Social Media</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>18 tasks x 4 voices x 3 platforms + format playbook + weekly cadence</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Carl Agent Spec v2.0</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Docx</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/FAdydmo4FosxDSxT9vTcLMQpnph</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Agent Specs</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Updated to reflect dual role: WAVE build + Content/Flywheel ops</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Social Content Tracker v1.1</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Excel (file)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/ZFgAbmdwwoPfbZxKj5JcKpZLnIh</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>5 sheets — tracker, format playbook, voice matrix, weekly cadence, summary. 26 tasks, 17 formats, 4 voices + Emily ops</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Social Content Operations Playbook v1.1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Docx (file)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/Awl4bydJIo6rQdxs7hAcBD8zn7N</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Full social strategy — 3 platforms, 4 voices, 17 formats, 7-dimension brand guardrails, repurposing pyramid, B2B differentiation research integrated</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Emily — Social Content Onboarding Guide</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Docx (file)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/P8mzbaZFYofCaMxNU0bck7Oynae</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Onboarding guide for Emily — role scope, deliverables, brand guardrails, weekly rhythm, quality checklist, first-week action plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Carl Agent Spec v2.0</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Docx</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/FAdydmo4FosxDSxT9vTcLMQpnph</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Agent Spec</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Dual role: WAVE build + Content/Flywheel operations. 10 chapters.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4710,6 +4285,1124 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="53" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Document Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Feishu Link</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Content Pillar</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Content Pillars Aligned v3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/sheets/VDkPsNGEwhmLa4tqA9pcatHNnEh</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Content Calendar</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Master calendar - 3 webinars/mo + workshops by pillar</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Headline-First System v2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/sheets/OBsMsiX4ThazS1t3ZveczT9inrh</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Content System</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>15 hooks x 3 formats (long/short/reel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Week 1 Scripts v2</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/D2dBdUYMyoIaJSxwULvcR4cFnkd</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>ECHO v4.0 compliant</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>45 scripts (15 hooks x 3), ~22,403 words</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Series A v7</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/Jq8wdU4xloiJAmxHy1wcIDp4n7d</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>18 hooks, 54 scripts</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Series B v8</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/VYcZdgCOCoh6hgxQjRFc8lvKnjd</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Tone revised</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>24 hooks, 72 scripts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Series C Hook Map v7</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/LvWqd4514oBRK7xKmx4c3dX9nZe</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hook Map</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>China &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>25 hooks, 5 clusters</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Series C Sample Scripts v9</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/ZuCIdAQEDoyeiQxmwoGcdXtanJV</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>China &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>4 samples done</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>4 sample scripts; full 75 pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Series D Hook Map v10</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/VpFJdD1iQoPO9Lxt86Ic8QKpn4e</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hook Map</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>25 hooks, 5 clusters</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Series D Sample Scripts v10</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/VabodDdjJo9eO8xRGFEcrFe6nbc</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Scripts</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>4 samples done</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>4 sample scripts; full 75 pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Content Calendar v1 (legacy)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/sheets/XgKrsJNJyhiq6At2ebxc62IAnFR</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Content Calendar</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Superseded by v3</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Original calendar before pillar alignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>WAVE BRD v1.0</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/NsrodeH2doEWwMx67fCcT8Xtncc</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Business Requirements Document - 8 modules, 87 tickets</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>WAVE Development Tickets v1.0</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/OLuLdFDWdofvXzxRYCWce2gXnGd</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>87 dev tickets with priority/effort/deps</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>WAVE Intelligence Layer Spec v1.0</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/AqQSdPFxMoXmsyx1LRbcVqAgnqb</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Intelligence module specification</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>LYC Intelligence Design Spec</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/JaczdojEQo7NCBxeoqJco2Ylnod</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Intelligence design specification</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Outreach Funnel Refined v2</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/KNjedt5jsoUWkfxF7Q1cJL8jnuf</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Outreach funnel v2 refined spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Outreach Funnel Mapping Spec</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/PyYPdvoj5oy80FxZgPOcpUhNn5d</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Outreach funnel mapping specification</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>WAVE DB Schema - Outreach Funnel</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/CcQTdIh8FoO5YqxKpUXcvSS4n5b</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>App Spec</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Database schema SQL for outreach funnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>WAVE Project PM Tracker</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>(uploaded file - GaHfbAhjPoF0Z5xUX49ca0mLnnM)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>87 tickets with status/priority/module tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>WAVE Business Spec Pitch ICP</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Slides</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>(uploaded file - Qye0bsFr5oNzEDx6Oq4c8gnunHg)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>WAVE</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Business pitch deck for ICP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>ECHO Asset Master v6.0</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Doc (Notion)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://lyc-partners.notion.site/ECHO-Asset-Master-v6-0-Source-of-Truth-2026-08-04-3b2fafae51be81aeb291ec9c33e67faa</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Brand Compliance</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Echo</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Source of Truth</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Brand compliance source of truth - designated by Kevin 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Social Content Tracker v1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>File (xlsx)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/Nmu4bW4SCoxjjcxMo5pca1N3nPg</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Social Media</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>18 tasks x 4 voices x 3 platforms + format playbook + weekly cadence</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Carl Agent Spec v2.0</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Docx</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/FAdydmo4FosxDSxT9vTcLMQpnph</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Agent Specs</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Updated to reflect dual role: WAVE build + Content/Flywheel ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Social Content Tracker v1.1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Excel (file)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/ZFgAbmdwwoPfbZxKj5JcKpZLnIh</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>5 sheets — tracker, format playbook, voice matrix, weekly cadence, summary. 26 tasks, 17 formats, 4 voices + Emily ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Social Content Operations Playbook v1.1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Docx (file)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/Awl4bydJIo6rQdxs7hAcBD8zn7N</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Full social strategy — 3 platforms, 4 voices, 17 formats, 7-dimension brand guardrails, repurposing pyramid, B2B differentiation research integrated</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Emily — Social Content Onboarding Guide</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Docx (file)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/P8mzbaZFYofCaMxNU0bck7Oynae</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Content Operations</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Onboarding guide for Emily — role scope, deliverables, brand guardrails, weekly rhythm, quality checklist, first-week action plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Carl Agent Spec v2.0</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Docx</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/FAdydmo4FosxDSxT9vTcLMQpnph</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Agent Spec</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Dual role: WAVE build + Content/Flywheel operations. 10 chapters.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5814,7 +6507,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6294,7 +6987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6643,7 +7336,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7648,7 +8341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8142,697 +8835,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="53" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>File Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Path</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>webinar_definitions.json</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Event Data</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>29 industry x geo webinar cluster definitions</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>webinar_programs.json</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Event Data</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Program definitions with matching rules, tier assignments</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Automation_Spec_v1.md</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Spec</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Automation specification for Carl workflows</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Density_Clustering_Report_v1.md</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Contact density clustering analysis</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Density_Clustering_Report_v2.md</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Updated density clustering</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Cross_Cluster_Mapping_Report_v1.md</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Cross-cluster contact mapping</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Strategic_Priority_DeepDive_v1.md</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Strategic priority deep-dive</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Subsegmentation_Report_v1.md</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Report</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Contact subsegmentation analysis</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>LYC_Content_Pillars_Aligned_v2.xlsx</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Calendar</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Source Excel for Feishu Content Pillars v3</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>LYC_WEEK1_SCRIPTS_V2_FULL.md</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Week 1 v2 complete scripts (~22,403 words)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>headline_scripts_v2_final.json</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Week 1 v2 scripts JSON</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>LYC_YOUTUBE_SCRIPTS_V7_ALL_18_HOOKS_COMPLETE.md</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Series A complete scripts</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>LYC_YOUTUBE_V8_TONE_REVISED.md</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Scripts</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Series B complete scripts</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>LYC_YOUTUBE_HOOK_MAP_V7_BEYOND_HEADLINES.md</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Hook Map</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Series C hook map</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>LYC_YOUTUBE_HOOK_MAP_V10_AI_CAREER.md</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hook Map</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Series D hook map</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Full_Inventory.md</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Complete Carl asset inventory (Markdown)</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CARL_Supabase_Tables_Spec.md</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Supabase table specs + workflows</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>WAVE_Project_PM_Tracker.xlsx</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>PM Tracker</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>WAVE project management - 87 tickets with status</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>WAVE_Project/Business_Specs/</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>App Spec</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>WAVE business specs (BRD, tickets, intelligence, funnel)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>WAVE_Project/Database_Schema/</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>DB Schema</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Outreach funnel SQL schema</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>WAVE_Project/wave-app/</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Source Code</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Next.js source code for WAVE app (Phase 0)</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>LYC_Social_Content_Tracker_v1.xlsx</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Social Media Tracker</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>./</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>LYC_Social_Content_Tracker_v1.1.xlsx</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Social content tracker — 5 sheets, 26 tasks, 17 formats</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>social_content_playbook_v1.1.docx</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Full social playbook v1.1 with B2B differentiation research</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>emily_social_content_onboarding.docx</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Content Operations</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Emily onboarding guide</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>carl_agent_spec_v2.docx</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Agent Identity</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Carl agent spec v2 — dual role (WAVE + content ops)</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>/app/data/sessions/session/</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Comms Methodology sheet (Sheet 9 from Unified Strategy Tracker)
</commit_message>
<xml_diff>
--- a/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
+++ b/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
@@ -9,15 +9,16 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Rollout" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Webinar #1 Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEXUS Board Strategy Comm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feishu Files" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comms Methodology" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NEXUS Board Strategy Comm" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feishu Files" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notion Pages" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supabase Tables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apps &amp; Platforms" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specs &amp; Documents" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Pipeline" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local Files" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,8 +104,32 @@
       <color rgb="00D4AC0D"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00833C0C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -195,8 +220,44 @@
         <bgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+        <bgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -252,11 +313,25 @@
         <color rgb="00E0E2E6"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4C7E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4C7E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C7E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C7E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -324,6 +399,22 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="15" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2075,6 +2166,502 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="53" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Series</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Perspective</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Content Pillar</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Hooks</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Scripts Done</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Scripts Total</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Feishu Link</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Series A (v7)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>I've lived this</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/Jq8wdU4xloiJAmxHy1wcIDp4n7d</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Series B (v8)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>I've watched from the chair</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/VYcZdgCOCoh6hgxQjRFc8lvKnjd</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Tone revised</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Series C (v9)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>I've placed them across both worlds</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>China &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/LvWqd4514oBRK7xKmx4c3dX9nZe</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hook map + 4 samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Series D (v10)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>I see who's ready</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/VpFJdD1iQoPO9Lxt86Ic8QKpn4e</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Hook map + 4 samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Week 1 v2 (cross-series)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/docx/D2dBdUYMyoIaJSxwULvcR4cFnkd</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>ECHO v4.0 compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Headline-First System v2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/sheets/OBsMsiX4ThazS1t3ZveczT9inrh</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Social Content (Multi-platform)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Podcast/webinar repurpose + original</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>12 formats</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>~15 posts/week target</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/Nmu4bW4SCoxjjcxMo5pca1N3nPg</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Just started - v1 tracker live</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Social Content — LinkedIn 4 Voices</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4-voice triangulation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/ZFgAbmdwwoPfbZxKj5JcKpZLnIh</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Onboarding — Week of Aug 11 start</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Social Content — Instagram</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Editorial premium aesthetic</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Starting with Kevin/brand account</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Social Content — YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Repurposing layer only</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>All 3 Pillars</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>3-4/week — search-optimized, from long-form only</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2762,7 +3349,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3889,6 +4476,552 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Comms Methodology — Agency Pitch Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Phased, decision-gated approach to product communication strategy — from the NEXUS GTM process</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Core Principles (5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Principle</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Taxonomy Principle</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="inlineStr">
+        <is>
+          <t>Outcomes lead. Methods follow. Taxonomy recedes. Users should know what they're getting and why before they learn internal framework names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Decision Gates, Not Revisions</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>Each phase ends with a lock. Once locked, it doesn't reopen unless new information changes the underlying assumption. Prevents scope drift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Anti-Positioning First</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>You don't win by saying you're better. You win by changing the frame of the comparison. Define who you're positioning against and how you reframe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>One Engine, Many Voices</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Every core idea propagates across voices and channels. Strategy defines who says what, where, and to what end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>The Product Never Speaks First</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>Thought leader builds the category. Product voice explains the solution. Institutional voice closes enterprise sale. Nobody feels sold to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Phase Overview (6 Phases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>What Gets Decided</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>Brand Strategy &amp; Positioning</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Category, brand architecture, voice, tagline, visual system</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>Messaging Architecture &amp; Content Strategy</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>Message layers, audience messaging, anti-positioning, content pillars, content engine, objections</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>2-3 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>Launch Strategy &amp; Campaign Architecture</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>Launch timeline, campaign phases, content calendar, asset inventory</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Partnerships, Ecosystem &amp; KPI Framework</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Partner strategy, ecosystem integration, pricing tiers, KPIs, measurement plan</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>1-2 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Cross-Business Handoff (Optional)</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>How product feeds other business units (B2C→B2B, product→services)</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>Unified Flywheel Integration (Optional)</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>How product plugs into broader business flywheel — asset mapping, calendar, new North Star</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>1 day</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Common Pitfalls to Avoid (6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Pitfall</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>Why It's a Problem</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>Skipping Phase 1</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>Everyone wants to talk about launch tactics. Positioning is 80% of the work. Get it right first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
+        <is>
+          <t>Doing everything in one meeting</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>The brain can only absorb so much. One phase at a time. One decision at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>Revisiting locked decisions</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>"I just had another idea" is not new information. New competitor or market data? That's a reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>Leading with taxonomy</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Resist showing off frameworks and clever names. Audience doesn't care what you call it. They care what it does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>Forgetting anti-positioning</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Every category has incumbents. If you don't define how you're different, people default to price and features.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>No North Star metric</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>If you don't know what winning looks like, you'll never know if you won. Pick one thing. Measure it obsessively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>Application to LYC Brand Rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>Methodology Element</t>
+        </is>
+      </c>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>How It's Applied in Rollout</t>
+        </is>
+      </c>
+      <c r="C31" s="34" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>Taxonomy Principle</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>All content leads with outcomes (what you get), not framework names. ECHO enforces across all assets.</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="inlineStr">
+        <is>
+          <t>ECHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>Decision Gates</t>
+        </is>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>Each Phase of the brand rollout has explicit lock points. Kevin signs off before moving forward.</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="inlineStr">
+        <is>
+          <t>Kevin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>Anti-Positioning</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>LYC positions against legacy retainer search firms — frame reframed as intelligence vs. staffing.</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>Kevin / ECHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t>One Engine, Many Voices</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>4 LinkedIn profiles (Kevin/Claire/Jaelyn/Joyce) share one thesis, each from a different angle.</t>
+        </is>
+      </c>
+      <c r="C35" s="32" t="inlineStr">
+        <is>
+          <t>ECHO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>Product Never Speaks First</t>
+        </is>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Kevin's thought leadership builds the category first; Claire's product content explains solutions.</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>Kevin / Claire</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>6-Phase Model</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>LYC brand rollout follows the same 6 phases, compressed into a 1-week sprint with decision gates.</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>North Star Metric</t>
+        </is>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>Webinar #1 registrations (Aug 19) serve as the launch-phase North Star.</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>LENS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4279,7 +5412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5397,7 +6530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6507,7 +7640,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6987,7 +8120,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7336,7 +8469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8339,500 +9472,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="53" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Series</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Perspective</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Content Pillar</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Total Hooks</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Scripts Done</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Scripts Total</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Feishu Link</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Series A (v7)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>I've lived this</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Career</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/Jq8wdU4xloiJAmxHy1wcIDp4n7d</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Series B (v8)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>I've watched from the chair</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Career</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/VYcZdgCOCoh6hgxQjRFc8lvKnjd</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Tone revised</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Series C (v9)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>I've placed them across both worlds</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>China &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/LvWqd4514oBRK7xKmx4c3dX9nZe</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Hook map + 4 samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Series D (v10)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>I see who's ready</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>AI &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/VpFJdD1iQoPO9Lxt86Ic8QKpn4e</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Hook map + 4 samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Week 1 v2 (cross-series)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/docx/D2dBdUYMyoIaJSxwULvcR4cFnkd</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>ECHO v4.0 compliant</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Headline-First System v2</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/sheets/OBsMsiX4ThazS1t3ZveczT9inrh</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Social Content (Multi-platform)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Podcast/webinar repurpose + original</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>12 formats</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>~15 posts/week target</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/Nmu4bW4SCoxjjcxMo5pca1N3nPg</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Just started - v1 tracker live</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Social Content — LinkedIn 4 Voices</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>4-voice triangulation</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://l5tf5m43wr.feishu.cn/file/ZFgAbmdwwoPfbZxKj5JcKpZLnIh</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Onboarding — Week of Aug 11 start</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Social Content — Instagram</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Editorial premium aesthetic</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Starting with Kevin/brand account</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Social Content — YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Repurposing layer only</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>All 3 Pillars</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>3-4/week — search-optimized, from long-form only</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Feishu file reference to tracker sheet
</commit_message>
<xml_diff>
--- a/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
+++ b/brand-rollout/LYC_Master_Asset_Tracker_v4.xlsx
@@ -5418,7 +5418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6510,6 +6510,43 @@
       <c r="H27" t="inlineStr">
         <is>
           <t>Dual role: WAVE build + Content/Flywheel operations. 10 chapters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LYC Master Asset Tracker (v5 - with Comms Meth)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EFyHbdDyQok7hAxNAa6cgygZntc</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Master tracker with comms methodology sheet integrated</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://l5tf5m43wr.feishu.cn/file/EFyHbdDyQok7hAxNAa6cgygZntc</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Aug 7, 2026</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>